<commit_message>
docs: README com funcionalidades, arquitetura e capturas de tela
</commit_message>
<xml_diff>
--- a/templates/planilha-financeira-exemplo.xlsx
+++ b/templates/planilha-financeira-exemplo.xlsx
@@ -1283,7 +1283,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4048B589-F4AD-4942-86E4-33BBC73BF143}</x14:id>
+          <x14:id>{E702CC5F-0C85-45B8-8D61-A0E9F8C0C492}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1294,7 +1294,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4048B589-F4AD-4942-86E4-33BBC73BF143}">
+          <x14:cfRule type="dataBar" id="{E702CC5F-0C85-45B8-8D61-A0E9F8C0C492}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
feat: adiciona categorias para motoristas de aplicativo
Inclui a receita "Aplicativos (Uber, 99, iFood)" e o gasto essencial
"Combustível", permitindo acompanhar o ganho líquido das corridas.
Modelos de planilha regenerados com as novas listas.
</commit_message>
<xml_diff>
--- a/templates/planilha-financeira-exemplo.xlsx
+++ b/templates/planilha-financeira-exemplo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="124">
   <si>
     <t>Resumo financeiro</t>
   </si>
@@ -59,60 +59,63 @@
     <t>Dívidas em aberto</t>
   </si>
   <si>
+    <t>Combustível</t>
+  </si>
+  <si>
+    <t>Juros das dívidas por mês</t>
+  </si>
+  <si>
     <t>Contas da casa</t>
   </si>
   <si>
-    <t>Juros das dívidas por mês</t>
+    <t>Parcelas de dívidas por mês</t>
   </si>
   <si>
     <t>Saúde</t>
   </si>
   <si>
-    <t>Parcelas de dívidas por mês</t>
+    <t>Comprometimento da renda</t>
   </si>
   <si>
     <t>Educação</t>
   </si>
   <si>
-    <t>Comprometimento da renda</t>
+    <t>Patrimônio investido</t>
   </si>
   <si>
     <t>Lazer</t>
   </si>
   <si>
-    <t>Patrimônio investido</t>
+    <t>Aportes planejados por mês</t>
   </si>
   <si>
     <t>Assinaturas</t>
   </si>
   <si>
-    <t>Aportes planejados por mês</t>
-  </si>
-  <si>
     <t>Vestuário</t>
   </si>
   <si>
+    <t>Últimos 12 meses</t>
+  </si>
+  <si>
     <t>Pagamento de dívidas</t>
   </si>
   <si>
-    <t>Últimos 12 meses</t>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Ganhos</t>
+  </si>
+  <si>
+    <t>Gastos</t>
+  </si>
+  <si>
+    <t>Saldo</t>
   </si>
   <si>
     <t>Investimentos</t>
   </si>
   <si>
-    <t>Mês</t>
-  </si>
-  <si>
-    <t>Ganhos</t>
-  </si>
-  <si>
-    <t>Gastos</t>
-  </si>
-  <si>
-    <t>Saldo</t>
-  </si>
-  <si>
     <t>Outros gastos</t>
   </si>
   <si>
@@ -369,6 +372,9 @@
   </si>
   <si>
     <t>Outro</t>
+  </si>
+  <si>
+    <t>Aplicativos (Uber, 99, iFood)</t>
   </si>
   <si>
     <t>Vendas</t>
@@ -1095,7 +1101,7 @@
         <f>IF($B$5=0,0,G16/$B$5)</f>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="10">
         <f>EDATE($B$2,-11)</f>
       </c>
@@ -1107,6 +1113,15 @@
       </c>
       <c r="D17" s="6">
         <f>B17-C17</f>
+      </c>
+      <c r="F17" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="6">
+        <f>SUMIFS('Lançamentos'!$E:$E,'Lançamentos'!$D:$D,"Gasto",'Lançamentos'!$A:$A,"&gt;="&amp;$B$2,'Lançamentos'!$A:$A,"&lt;="&amp;$C$2,'Lançamentos'!$C:$C,F17)</f>
+      </c>
+      <c r="H17" s="7">
+        <f>IF($B$5=0,0,G17/$B$5)</f>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1265,7 +1280,7 @@
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1274,7 +1289,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:H16">
+  <conditionalFormatting sqref="H4:H17">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1283,7 +1298,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E702CC5F-0C85-45B8-8D61-A0E9F8C0C492}</x14:id>
+          <x14:id>{8FC642ED-789C-49E9-83C8-B320982360D2}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1294,7 +1309,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E702CC5F-0C85-45B8-8D61-A0E9F8C0C492}">
+          <x14:cfRule type="dataBar" id="{8FC642ED-789C-49E9-83C8-B320982360D2}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -1304,7 +1319,7 @@
               </x14:cfvo>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>H4:H16</xm:sqref>
+          <xm:sqref>H4:H17</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -1330,22 +1345,22 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1353,19 +1368,19 @@
         <v>46147</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" s="6">
         <v>2150</v>
       </c>
       <c r="F2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1373,19 +1388,19 @@
         <v>46148</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E3" s="6">
         <v>750</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1393,19 +1408,19 @@
         <v>46149</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E4" s="6">
         <v>441</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1413,19 +1428,19 @@
         <v>46150</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" s="6">
         <v>181</v>
       </c>
       <c r="F5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1433,19 +1448,19 @@
         <v>46151</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" s="6">
         <v>120</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1453,19 +1468,19 @@
         <v>46152</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="6">
         <v>180</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1473,19 +1488,19 @@
         <v>46154</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E8" s="6">
         <v>200</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1493,19 +1508,19 @@
         <v>46157</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E9" s="6">
         <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1513,19 +1528,19 @@
         <v>46162</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E10" s="6">
         <v>180</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1533,19 +1548,19 @@
         <v>46163</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" s="6">
         <v>168</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1553,19 +1568,19 @@
         <v>46167</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E12" s="6">
         <v>95</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1573,19 +1588,19 @@
         <v>46169</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E13" s="6">
         <v>147</v>
       </c>
       <c r="F13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1593,19 +1608,19 @@
         <v>46178</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" s="6">
         <v>2150</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1613,19 +1628,19 @@
         <v>46179</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E15" s="6">
         <v>750</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1633,19 +1648,19 @@
         <v>46180</v>
       </c>
       <c r="B16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E16" s="6">
         <v>412</v>
       </c>
       <c r="F16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1653,19 +1668,19 @@
         <v>46181</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E17" s="6">
         <v>205</v>
       </c>
       <c r="F17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1673,19 +1688,19 @@
         <v>46182</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E18" s="6">
         <v>120</v>
       </c>
       <c r="F18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1693,19 +1708,19 @@
         <v>46183</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E19" s="6">
         <v>180</v>
       </c>
       <c r="F19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1713,19 +1728,19 @@
         <v>46185</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E20" s="6">
         <v>227</v>
       </c>
       <c r="F20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1733,19 +1748,19 @@
         <v>46188</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E21" s="6">
         <v>65</v>
       </c>
       <c r="F21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1753,19 +1768,19 @@
         <v>46191</v>
       </c>
       <c r="B22" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" s="6">
         <v>378</v>
       </c>
       <c r="F22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1773,19 +1788,19 @@
         <v>46193</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E23" s="6">
         <v>180</v>
       </c>
       <c r="F23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1793,19 +1808,19 @@
         <v>46194</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C24" t="s">
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E24" s="6">
         <v>157</v>
       </c>
       <c r="F24" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1813,19 +1828,19 @@
         <v>46198</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E25" s="6">
         <v>95</v>
       </c>
       <c r="F25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1833,19 +1848,19 @@
         <v>46200</v>
       </c>
       <c r="B26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C26" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E26" s="6">
         <v>137</v>
       </c>
       <c r="F26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1853,19 +1868,19 @@
         <v>46208</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D27" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E27" s="6">
         <v>2150</v>
       </c>
       <c r="F27" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1873,19 +1888,19 @@
         <v>46209</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E28" s="6">
         <v>750</v>
       </c>
       <c r="F28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1893,19 +1908,19 @@
         <v>46210</v>
       </c>
       <c r="B29" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C29" t="s">
         <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E29" s="6">
         <v>382</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1913,19 +1928,19 @@
         <v>46211</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C30" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E30" s="6">
         <v>192</v>
       </c>
       <c r="F30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1933,19 +1948,19 @@
         <v>46212</v>
       </c>
       <c r="B31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E31" s="6">
         <v>120</v>
       </c>
       <c r="F31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -1953,19 +1968,19 @@
         <v>46213</v>
       </c>
       <c r="B32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E32" s="6">
         <v>180</v>
       </c>
       <c r="F32" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1973,19 +1988,19 @@
         <v>46215</v>
       </c>
       <c r="B33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C33" t="s">
         <v>8</v>
       </c>
       <c r="D33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E33" s="6">
         <v>212</v>
       </c>
       <c r="F33" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -1993,19 +2008,19 @@
         <v>46218</v>
       </c>
       <c r="B34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C34" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E34" s="6">
         <v>65</v>
       </c>
       <c r="F34" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -2013,19 +2028,19 @@
         <v>46223</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C35" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D35" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E35" s="6">
         <v>180</v>
       </c>
       <c r="F35" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -2033,19 +2048,19 @@
         <v>46224</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C36" t="s">
         <v>10</v>
       </c>
       <c r="D36" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E36" s="6">
         <v>146</v>
       </c>
       <c r="F36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -2053,19 +2068,19 @@
         <v>46228</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C37" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D37" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E37" s="6">
         <v>95</v>
       </c>
       <c r="F37" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -2073,19 +2088,19 @@
         <v>46230</v>
       </c>
       <c r="B38" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C38" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E38" s="6">
         <v>127</v>
       </c>
       <c r="F38" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -2093,19 +2108,19 @@
         <v>46239</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D39" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E39" s="6">
         <v>2150</v>
       </c>
       <c r="F39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -2113,19 +2128,19 @@
         <v>46240</v>
       </c>
       <c r="B40" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
       </c>
       <c r="D40" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E40" s="6">
         <v>750</v>
       </c>
       <c r="F40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2133,19 +2148,19 @@
         <v>46241</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s">
         <v>10</v>
       </c>
       <c r="D41" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E41" s="6">
         <v>437</v>
       </c>
       <c r="F41" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -2153,19 +2168,19 @@
         <v>46242</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C42" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D42" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E42" s="6">
         <v>179</v>
       </c>
       <c r="F42" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -2173,19 +2188,19 @@
         <v>46243</v>
       </c>
       <c r="B43" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C43" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D43" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E43" s="6">
         <v>120</v>
       </c>
       <c r="F43" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2193,19 +2208,19 @@
         <v>46244</v>
       </c>
       <c r="B44" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
       </c>
       <c r="D44" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E44" s="6">
         <v>180</v>
       </c>
       <c r="F44" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -2213,19 +2228,19 @@
         <v>46246</v>
       </c>
       <c r="B45" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C45" t="s">
         <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E45" s="6">
         <v>197</v>
       </c>
       <c r="F45" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -2233,19 +2248,19 @@
         <v>46248</v>
       </c>
       <c r="B46" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C46" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D46" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E46" s="6">
         <v>86</v>
       </c>
       <c r="F46" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -2253,19 +2268,19 @@
         <v>46249</v>
       </c>
       <c r="B47" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D47" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E47" s="6">
         <v>65</v>
       </c>
       <c r="F47" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -2273,19 +2288,19 @@
         <v>46252</v>
       </c>
       <c r="B48" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D48" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E48" s="6">
         <v>329</v>
       </c>
       <c r="F48" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -2293,19 +2308,19 @@
         <v>46254</v>
       </c>
       <c r="B49" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C49" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D49" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E49" s="6">
         <v>180</v>
       </c>
       <c r="F49" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -2313,19 +2328,19 @@
         <v>46255</v>
       </c>
       <c r="B50" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C50" t="s">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E50" s="6">
         <v>166</v>
       </c>
       <c r="F50" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -2333,19 +2348,19 @@
         <v>46259</v>
       </c>
       <c r="B51" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C51" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D51" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E51" s="6">
         <v>95</v>
       </c>
       <c r="F51" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2353,19 +2368,19 @@
         <v>46261</v>
       </c>
       <c r="B52" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C52" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E52" s="6">
         <v>146</v>
       </c>
       <c r="F52" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -2373,19 +2388,19 @@
         <v>46270</v>
       </c>
       <c r="B53" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C53" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D53" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E53" s="6">
         <v>2150</v>
       </c>
       <c r="F53" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -2393,19 +2408,19 @@
         <v>46271</v>
       </c>
       <c r="B54" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C54" t="s">
         <v>6</v>
       </c>
       <c r="D54" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E54" s="6">
         <v>750</v>
       </c>
       <c r="F54" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -2413,19 +2428,19 @@
         <v>46272</v>
       </c>
       <c r="B55" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C55" t="s">
         <v>10</v>
       </c>
       <c r="D55" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E55" s="6">
         <v>407</v>
       </c>
       <c r="F55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -2433,19 +2448,19 @@
         <v>46273</v>
       </c>
       <c r="B56" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C56" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D56" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E56" s="6">
         <v>203</v>
       </c>
       <c r="F56" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -2453,19 +2468,19 @@
         <v>46274</v>
       </c>
       <c r="B57" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C57" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D57" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E57" s="6">
         <v>120</v>
       </c>
       <c r="F57" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -2473,19 +2488,19 @@
         <v>46275</v>
       </c>
       <c r="B58" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C58" t="s">
         <v>12</v>
       </c>
       <c r="D58" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E58" s="6">
         <v>180</v>
       </c>
       <c r="F58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -2493,19 +2508,19 @@
         <v>46277</v>
       </c>
       <c r="B59" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E59" s="6">
         <v>225</v>
       </c>
       <c r="F59" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2513,19 +2528,19 @@
         <v>46280</v>
       </c>
       <c r="B60" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C60" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D60" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E60" s="6">
         <v>65</v>
       </c>
       <c r="F60" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -2533,19 +2548,19 @@
         <v>46285</v>
       </c>
       <c r="B61" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D61" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E61" s="6">
         <v>180</v>
       </c>
       <c r="F61" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -2553,19 +2568,19 @@
         <v>46286</v>
       </c>
       <c r="B62" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C62" t="s">
         <v>10</v>
       </c>
       <c r="D62" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E62" s="6">
         <v>155</v>
       </c>
       <c r="F62" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2573,19 +2588,19 @@
         <v>46290</v>
       </c>
       <c r="B63" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C63" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D63" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E63" s="6">
         <v>95</v>
       </c>
       <c r="F63" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2593,19 +2608,19 @@
         <v>46292</v>
       </c>
       <c r="B64" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C64" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D64" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E64" s="6">
         <v>136</v>
       </c>
       <c r="F64" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -2613,19 +2628,19 @@
         <v>46298</v>
       </c>
       <c r="B65" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C65" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D65" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E65" s="6">
         <v>50</v>
       </c>
       <c r="F65" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2633,19 +2648,19 @@
         <v>46300</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C66" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D66" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E66" s="6">
         <v>2150</v>
       </c>
       <c r="F66" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2653,19 +2668,19 @@
         <v>46301</v>
       </c>
       <c r="B67" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C67" t="s">
         <v>6</v>
       </c>
       <c r="D67" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E67" s="6">
         <v>750</v>
       </c>
       <c r="F67" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2673,19 +2688,19 @@
         <v>46302</v>
       </c>
       <c r="B68" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C68" t="s">
         <v>10</v>
       </c>
       <c r="D68" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E68" s="6">
         <v>378</v>
       </c>
       <c r="F68" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2693,19 +2708,19 @@
         <v>46303</v>
       </c>
       <c r="B69" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C69" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D69" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E69" s="6">
         <v>190</v>
       </c>
       <c r="F69" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2713,19 +2728,19 @@
         <v>46304</v>
       </c>
       <c r="B70" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C70" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D70" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E70" s="6">
         <v>120</v>
       </c>
       <c r="F70" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2733,19 +2748,19 @@
         <v>46305</v>
       </c>
       <c r="B71" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C71" t="s">
         <v>12</v>
       </c>
       <c r="D71" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E71" s="6">
         <v>180</v>
       </c>
       <c r="F71" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2753,19 +2768,19 @@
         <v>46307</v>
       </c>
       <c r="B72" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C72" t="s">
         <v>8</v>
       </c>
       <c r="D72" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E72" s="6">
         <v>210</v>
       </c>
       <c r="F72" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2773,19 +2788,19 @@
         <v>46310</v>
       </c>
       <c r="B73" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C73" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D73" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E73" s="6">
         <v>65</v>
       </c>
       <c r="F73" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2793,19 +2808,19 @@
         <v>46313</v>
       </c>
       <c r="B74" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C74" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D74" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E74" s="6">
         <v>350</v>
       </c>
       <c r="F74" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -2813,19 +2828,19 @@
         <v>46315</v>
       </c>
       <c r="B75" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C75" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D75" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E75" s="6">
         <v>180</v>
       </c>
       <c r="F75" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -2833,19 +2848,19 @@
         <v>46316</v>
       </c>
       <c r="B76" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C76" t="s">
         <v>10</v>
       </c>
       <c r="D76" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E76" s="6">
         <v>144</v>
       </c>
       <c r="F76" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -2853,19 +2868,19 @@
         <v>46320</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C77" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D77" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E77" s="6">
         <v>95</v>
       </c>
       <c r="F77" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2873,19 +2888,19 @@
         <v>46322</v>
       </c>
       <c r="B78" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C78" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E78" s="6">
         <v>126</v>
       </c>
       <c r="F78" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="79" spans="3:6" x14ac:dyDescent="0.25"/>
@@ -3815,10 +3830,10 @@
   <autoFilter ref="A1:F1"/>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C10:C1001">
-      <formula1>Listas!$B$2:$B$20</formula1>
+      <formula1>Listas!$B$2:$B$22</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1001">
-      <formula1>Listas!$B$2:$B$20</formula1>
+      <formula1>Listas!$B$2:$B$22</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D10:D1001">
       <formula1>Listas!$A$2:$A$3</formula1>
@@ -3860,42 +3875,42 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="6">
         <v>3200</v>
@@ -3913,21 +3928,21 @@
         <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I2" s="6">
         <f>IF(C2="","",C2*D2/100)</f>
       </c>
       <c r="J2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" s="6">
         <v>650</v>
@@ -3945,7 +3960,7 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I3" s="6">
         <f>IF(C3="","",C3*D3/100)</f>
@@ -3953,10 +3968,10 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C4" s="6">
         <v>780</v>
@@ -3974,7 +3989,7 @@
         <v>25</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I4" s="6">
         <f>IF(C4="","",C4*D4/100)</f>
@@ -3982,10 +3997,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" s="6">
         <v>1400</v>
@@ -4003,13 +4018,13 @@
         <v>10</v>
       </c>
       <c r="H5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I5" s="6">
         <f>IF(C5="","",C5*D5/100)</f>
       </c>
       <c r="J5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -4426,51 +4441,51 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K1" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2" s="6">
         <v>150</v>
@@ -4497,18 +4512,18 @@
         <v>46237</v>
       </c>
       <c r="L2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D3" s="6">
         <v>0</v>
@@ -4535,18 +4550,18 @@
         <v>46539</v>
       </c>
       <c r="L3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" s="6">
         <v>0</v>
@@ -4971,7 +4986,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="26" customWidth="1"/>
@@ -4979,71 +4994,71 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
@@ -5051,13 +5066,13 @@
         <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
@@ -5065,13 +5080,13 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
@@ -5079,13 +5094,13 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
@@ -5093,13 +5108,13 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
@@ -5107,10 +5122,10 @@
         <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
@@ -5118,7 +5133,7 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
@@ -5126,7 +5141,7 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
@@ -5134,7 +5149,7 @@
         <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
@@ -5154,22 +5169,22 @@
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
@@ -5180,6 +5195,16 @@
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>